<commit_message>
changes on LoginDDT Test
</commit_message>
<xml_diff>
--- a/Testdata/Opencart_LoginData.xlsx
+++ b/Testdata/Opencart_LoginData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DILIP KUMAR\eclipse-workspace\OpencartV\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB95DCAE-01A8-43B7-8BD0-729C983399D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0D62F7-5B39-4A80-836D-71CE9B98E29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1F2D179E-37D2-4BC0-88A9-F5C135B87DA5}"/>
   </bookViews>
@@ -538,7 +538,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.35">
@@ -571,7 +571,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="21" x14ac:dyDescent="0.35">

</xml_diff>